<commit_message>
redesign driver scanner ui
</commit_message>
<xml_diff>
--- a/.codex-tmp/rmr-plant-xlsx/output/SUEA_Safety_API_Inventory.xlsx
+++ b/.codex-tmp/rmr-plant-xlsx/output/SUEA_Safety_API_Inventory.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Summary" sheetId="1" r:id="R3e12936876c64d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_API_Inventory" sheetId="2" r:id="R456d1015e98e45d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Checkin_Locations" sheetId="3" r:id="R4d90e715f2a34d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Safety_Effort" sheetId="4" r:id="Rdc54cc0632924210"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Safety_Culture" sheetId="5" r:id="Rd6149dfc07bf48c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Uploads_Media" sheetId="6" r:id="Rade1f15d6f8944d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Table_Mapping" sheetId="7" r:id="R699245a09da94b6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Payload_Response" sheetId="8" r:id="R7442b8c89ae342b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Scale_Rules" sheetId="9" r:id="Re77241efbba3496e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Backlog" sheetId="10" r:id="R3ac98fa9b46744df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_API_Counts" sheetId="11" r:id="Rb330729848ef44fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Summary" sheetId="1" r:id="R805a135cf29242a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_API_Inventory" sheetId="2" r:id="Re3500e4d27b240db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Checkin_Locations" sheetId="3" r:id="R820674c7670341f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Safety_Effort" sheetId="4" r:id="R485fff4b8d044e99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Safety_Culture" sheetId="5" r:id="Rf93f845988004b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Uploads_Media" sheetId="6" r:id="Rbb441ddfd27d44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Table_Mapping" sheetId="7" r:id="Rc6390266ba434255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Payload_Response" sheetId="8" r:id="Rb6ae854fe1a3498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Scale_Rules" sheetId="9" r:id="R54bdd13627244530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Backlog" sheetId="10" r:id="R72dd7d25b86e452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_API_Counts" sheetId="11" r:id="Rbeecddf81325478c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -378,16 +378,16 @@
         <x:v>Backend structure</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>Next.js API routes + backend/components</x:v>
+        <x:v>API catalog 159 routes ต่อ backend/components และฐานจริง</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
-        <x:v>จัด src/app/api เป็น HTTP layer และ logic ใน backend/components/*</x:v>
+        <x:v>คง HTTP layer บางและแยก repository/persistence ตาม feature</x:v>
       </x:c>
       <x:c r="D2" s="10" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="E2" s="4" t="str">
-        <x:v>logic กระจายถ้า API เยอะขึ้น</x:v>
+        <x:v>ต้องทดสอบสิทธิ์ด้วย session จริง</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -395,7 +395,7 @@
         <x:v>Auth</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>SSO routes มีแล้ว</x:v>
+        <x:v>SSO/session/users ต่อฐานจริงแล้ว และแก้ profile_image_url เกินความยาว</x:v>
       </x:c>
       <x:c r="C3" s="4" t="str">
         <x:v>ใช้ session guard เดียวกันทุก API</x:v>
@@ -404,7 +404,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
-        <x:v>สิทธิ์ admin/user ต้องชัด</x:v>
+        <x:v>ต้อง monitor callback และ schema drift</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -412,16 +412,16 @@
         <x:v>Locations</x:v>
       </x:c>
       <x:c r="B4" s="4" t="str">
-        <x:v>มี locations repository/API และ RMR SSO Plant sync design</x:v>
+        <x:v>Locations/Plant mirror/Admin CRUD ต่อฐานจริงแล้ว</x:v>
       </x:c>
       <x:c r="C4" s="4" t="str">
-        <x:v>rmr_sso.Plant read-only → mirror CPAC; Admin Plant เก็บ source=ADMIN</x:v>
+        <x:v>rmr_sso.Plant read-only → CPAC mirror; Admin Plant source=ADMIN</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
-        <x:v>ห้าม query ข้ามฐานทุก request และห้ามเขียน Plant Master</x:v>
+        <x:v>RMR source ห้ามแก้/ลบ</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -429,16 +429,16 @@
         <x:v>Check-in</x:v>
       </x:c>
       <x:c r="B5" s="4" t="str">
-        <x:v>UI มี mock/preset และ local state</x:v>
+        <x:v>หน้า Check-in โหลด locations และ POST checkins จริง</x:v>
       </x:c>
       <x:c r="C5" s="4" t="str">
-        <x:v>POST /api/checkins + history/admin list</x:v>
+        <x:v>ใช้ CPAC local location id และ GPS จริง</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
-        <x:v>ยังไม่ persist จริง</x:v>
+        <x:v>ต้องได้รับสิทธิ์ geolocation</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -446,16 +446,16 @@
         <x:v>Safety Effort</x:v>
       </x:c>
       <x:c r="B6" s="4" t="str">
-        <x:v>หลาย flow ยังอยู่ localStorage</x:v>
+        <x:v>Admin/Linewalk/Assessment ใช้ API และ feature tables จริง</x:v>
       </x:c>
       <x:c r="C6" s="4" t="str">
-        <x:v>activities, assessment-runs, reports, findings APIs</x:v>
+        <x:v>activities, runs, answers, findings/actions/comments</x:v>
       </x:c>
       <x:c r="D6" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
-        <x:v>รายงานจริง/รูปยังไม่พร้อม</x:v>
+        <x:v>ตรวจ workflow/permission รายบทบาท</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -463,16 +463,16 @@
         <x:v>Safety Culture</x:v>
       </x:c>
       <x:c r="B7" s="4" t="str">
-        <x:v>posts/events/rewards หลายส่วนอยู่ provider/localStorage</x:v>
+        <x:v>posts/events/rewards/teams/awareness ใช้ API และฐานจริง</x:v>
       </x:c>
       <x:c r="C7" s="4" t="str">
-        <x:v>posts/comments/reactions/events/rewards APIs</x:v>
+        <x:v>ไม่มี mock/localStorage ใน production flow</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>ข้อมูลหายข้ามเครื่อง</x:v>
+        <x:v>redeem ต้องอยู่ใน DB transaction</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -480,16 +480,16 @@
         <x:v>Media/images</x:v>
       </x:c>
       <x:c r="B8" s="4" t="str">
-        <x:v>base64/dataUrl ใน state/localStorage</x:v>
+        <x:v>uploads เก็บไฟล์จริงและ metadata ใน media_assets</x:v>
       </x:c>
       <x:c r="C8" s="4" t="str">
-        <x:v>object storage + media metadata + attachment IDs</x:v>
+        <x:v>owner_type/owner_id/link_type ผูกกับข้อมูลธุรกิจ</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E8" s="4" t="str">
-        <x:v>DB/browser/storage หนักถ้าใช้ base64</x:v>
+        <x:v>กำหนด storage retention และ access</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -497,16 +497,16 @@
         <x:v>Reports/export</x:v>
       </x:c>
       <x:c r="B9" s="4" t="str">
-        <x:v>localStorage + mock records</x:v>
+        <x:v>export_jobs เก็บสถานะและผลลัพธ์จริง</x:v>
       </x:c>
       <x:c r="C9" s="4" t="str">
-        <x:v>paginated report + async export</x:v>
+        <x:v>ดาวน์โหลดจาก job/result ไม่สร้าง mock response</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E9" s="4" t="str">
-        <x:v>ข้อมูลเยอะทำ timeout</x:v>
+        <x:v>งานใหญ่ควร background</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -514,7 +514,7 @@
         <x:v>Scale rules</x:v>
       </x:c>
       <x:c r="B10" s="4" t="str">
-        <x:v>limit บางเส้นมีแต่ยังไม่ครบ</x:v>
+        <x:v>list endpoints มี limit และ Plant อ่าน CPAC mirror</x:v>
       </x:c>
       <x:c r="C10" s="4" t="str">
         <x:v>pagination/bbox/index/cache ทุกเส้น list</x:v>
@@ -523,7 +523,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
-        <x:v>full scan/full payload</x:v>
+        <x:v>ติดตาม slow query</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -780,6 +780,57 @@
         <x:v>มี monitoring, retry และ import history</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="14" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>ย้าย feature JSON ออกจาก audit_logs</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>สร้าง 8 ตารางจริงและ migration แล้ว</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Backend/DB</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str">
+        <x:v>audit_logs เหลือ audit trail เท่านั้น</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="14" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>เชื่อมเมนูที่เปิดใช้งานกับ API จริง</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>Check-in, Safety Effort/Admin, Safety Culture, Notifications, Profile</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>ไม่มี business localStorage/mock fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="14" t="str">
+        <x:v>OUT OF SCOPE</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>Were OK / Work Permit</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>เมนูถูกปิดใน menu config</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="str">
+        <x:v>ไม่บังคับเชื่อม UI จนกว่าจะเปิดเมนู</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -804,10 +855,10 @@
         <x:v>Total API rows</x:v>
       </x:c>
       <x:c r="C1" s="9" t="str">
-        <x:v>Existing in repo</x:v>
+        <x:v>Existing/Connected</x:v>
       </x:c>
       <x:c r="D1" s="9" t="str">
-        <x:v>Target/New</x:v>
+        <x:v>Disabled menu</x:v>
       </x:c>
       <x:c r="E1" s="9" t="str">
         <x:v>Comment</x:v>
@@ -818,16 +869,16 @@
         <x:v>Safety Culture</x:v>
       </x:c>
       <x:c r="B2" s="4" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C2" s="4" t="n">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D2" s="4" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E2" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -844,7 +895,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
-        <x:v>Plant ใช้ CPAC mirror; RMR read-only และ Admin editable</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -855,13 +906,13 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="C4" s="4" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="n">
-        <x:v>11</x:v>
-      </x:c>
       <x:c r="E4" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -872,64 +923,64 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="n">
-        <x:v>9</x:v>
-      </x:c>
       <x:c r="E5" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="4" t="str">
-        <x:v>Check-in</x:v>
+        <x:v>Assessment</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D6" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="4" t="str">
-        <x:v>Safety Effort</x:v>
+        <x:v>Check-in</x:v>
       </x:c>
       <x:c r="B7" s="4" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>มีบางเส้นแล้วใน repo และมี target เพิ่ม</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="4" t="str">
-        <x:v>Assessment</x:v>
+        <x:v>Safety Effort</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C8" s="4" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D8" s="4" t="n">
-        <x:v>8</x:v>
-      </x:c>
       <x:c r="E8" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -940,13 +991,13 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C9" s="4" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D9" s="4" t="n">
-        <x:v>7</x:v>
-      </x:c>
       <x:c r="E9" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -957,30 +1008,30 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C10" s="4" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D10" s="4" t="n">
-        <x:v>7</x:v>
-      </x:c>
       <x:c r="E10" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="4" t="str">
-        <x:v>Organizations</x:v>
+        <x:v>Corrective Action</x:v>
       </x:c>
       <x:c r="B11" s="4" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C11" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="n">
-        <x:v>6</x:v>
-      </x:c>
       <x:c r="E11" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -991,115 +1042,115 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C12" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="n">
-        <x:v>6</x:v>
-      </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="4" t="str">
-        <x:v>Corrective Action</x:v>
+        <x:v>Organizations</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="n">
-        <x:v>6</x:v>
-      </x:c>
       <x:c r="E13" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="4" t="str">
-        <x:v>Safety Culture Admin</x:v>
+        <x:v>Rewards Admin</x:v>
       </x:c>
       <x:c r="B14" s="4" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C14" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D14" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="4" t="str">
-        <x:v>Rewards Admin</x:v>
+        <x:v>Safety Culture Admin</x:v>
       </x:c>
       <x:c r="B15" s="4" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C15" s="4" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="n">
-        <x:v>6</x:v>
-      </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="4" t="str">
-        <x:v>Uploads</x:v>
+        <x:v>Awareness Admin</x:v>
       </x:c>
       <x:c r="B16" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D16" s="4" t="n">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="E16" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="4" t="str">
-        <x:v>Awareness Admin</x:v>
+        <x:v>Media</x:v>
       </x:c>
       <x:c r="B17" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C17" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="n">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="E17" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="4" t="str">
-        <x:v>Media</x:v>
+        <x:v>Uploads</x:v>
       </x:c>
       <x:c r="B18" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D18" s="4" t="n">
-        <x:v>5</x:v>
-      </x:c>
       <x:c r="E18" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1116,7 +1167,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
-        <x:v>มีบางเส้นแล้วใน repo และมี target เพิ่ม</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1133,7 +1184,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>Backend route คงไว้ แต่เมนูปิดและไม่เชื่อม production UI</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1144,13 +1195,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C21" s="4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D21" s="4" t="n">
-        <x:v>3</x:v>
-      </x:c>
       <x:c r="E21" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1161,18 +1212,18 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D22" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="4" t="str">
-        <x:v>System</x:v>
+        <x:v>Settings</x:v>
       </x:c>
       <x:c r="B23" s="4" t="n">
         <x:v>2</x:v>
@@ -1184,41 +1235,41 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E23" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="4" t="str">
-        <x:v>Assistant</x:v>
+        <x:v>System</x:v>
       </x:c>
       <x:c r="B24" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C24" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D24" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E24" s="4" t="str">
-        <x:v>มีบางเส้นแล้วใน repo และมี target เพิ่ม</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="4" t="str">
-        <x:v>Awareness</x:v>
+        <x:v>Assistant</x:v>
       </x:c>
       <x:c r="B25" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C25" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D25" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="E25" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1229,30 +1280,47 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C26" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="E26" s="4" t="str">
-        <x:v>target design สำหรับ implement</x:v>
+        <x:v>API implementation มีใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="4" t="str">
+        <x:v>Awareness</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C27" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="4" t="str">
+        <x:v>API implementation มีใน repo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="14" t="str">
         <x:v>TOTAL</x:v>
       </x:c>
-      <x:c r="B27" s="4" t="n">
+      <x:c r="B28" s="14" t="n">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="n">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="C27" s="4" t="n">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="D27" s="4" t="n">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="E27" s="4" t="str">
-        <x:v>จำนวนเส้นใน inventory sheet</x:v>
+      <x:c r="D28" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>159 routes; active-menu routes connected</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1344,7 +1412,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K2" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>มีแล้วใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1379,7 +1447,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K3" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>มีแล้วใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1414,7 +1482,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K4" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>มีแล้วใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1434,7 +1502,7 @@
         <x:v>Header/Profile</x:v>
       </x:c>
       <x:c r="F5" s="4" t="str">
-        <x:v>เมื่อผู้ใช้เปิด logout endpoint</x:v>
+        <x:v>เมื่อกด logout</x:v>
       </x:c>
       <x:c r="G5" s="4" t="str">
         <x:v>User</x:v>
@@ -1449,7 +1517,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K5" s="4" t="str">
-        <x:v>มี dedicated route และล้าง session cookie</x:v>
+        <x:v>มีแล้วใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1484,7 +1552,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K6" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>มีแล้วใน repo</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1498,7 +1566,7 @@
         <x:v>/api/locations/plants</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>รายการโรงงานจาก CPAC mirror รวม RMR SSO Plant และ Admin Plant</x:v>
+        <x:v>รายการโรงงานสำหรับ check-in/search</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
         <x:v>Check-in, Admin</x:v>
@@ -1519,7 +1587,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
-        <x:v>อ่าน CPAC locations; คืน source, externalKey, readOnly; ไม่ query rmr_sso ทุก request</x:v>
+        <x:v>แยกจาก all locations เพราะข้อมูลเยอะ</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1743,7 +1811,7 @@
         <x:v>/api/locations</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:v>เพิ่ม location; ถ้า type=PLANT บังคับ source=ADMIN</x:v>
+        <x:v>เพิ่ม location ใหม่</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
         <x:v>Admin</x:v>
@@ -1764,7 +1832,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K14" s="4" t="str">
-        <x:v>เขียน CPAC_Safety.locations; Plant Admin ไม่เขียนกลับ rmr_sso.Plant</x:v>
+        <x:v>เขียนลง locations</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1778,7 +1846,7 @@
         <x:v>/api/locations/:id</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:v>แก้ไข location ที่ source อนุญาต</x:v>
+        <x:v>แก้ไข location</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
         <x:v>Admin</x:v>
@@ -1799,7 +1867,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K15" s="4" t="str">
-        <x:v>อนุญาต ADMIN/USER ตามสิทธิ์; RMR_SSO_PLANT ต้องตอบ 403 source_read_only</x:v>
+        <x:v>ต้อง audit</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1813,7 +1881,7 @@
         <x:v>/api/locations/:id</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:v>soft delete location ที่ source อนุญาต</x:v>
+        <x:v>soft delete location</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
         <x:v>Admin</x:v>
@@ -1834,7 +1902,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K16" s="4" t="str">
-        <x:v>อนุญาต ADMIN/USER ตามสิทธิ์; RMR_SSO_PLANT ต้องตอบ 403 source_read_only</x:v>
+        <x:v>soft delete เท่านั้น</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2216,7 +2284,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J27" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K27" s="4" t="str">
         <x:v>สร้าง safety_activities</x:v>
@@ -2251,7 +2319,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J28" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K28" s="4" t="str">
         <x:v>ใช้ resume draft/submitted</x:v>
@@ -2286,7 +2354,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J29" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K29" s="4" t="str">
         <x:v>เชื่อม checkin</x:v>
@@ -2321,7 +2389,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J30" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K30" s="4" t="str">
         <x:v>status draft/submitted/cancelled</x:v>
@@ -2356,7 +2424,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J31" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K31" s="4" t="str">
         <x:v>cache ได้</x:v>
@@ -2391,7 +2459,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J32" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K32" s="4" t="str">
         <x:v>payload ไม่ฝัง base64</x:v>
@@ -2426,7 +2494,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J33" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K33" s="4" t="str">
         <x:v>รวม answers + media refs</x:v>
@@ -2461,7 +2529,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J34" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K34" s="4" t="str">
         <x:v>export แยก endpoint</x:v>
@@ -2496,7 +2564,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J35" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K35" s="4" t="str">
         <x:v>สำหรับไฟล์ใหญ่ควรใช้ async job</x:v>
@@ -2531,7 +2599,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J36" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K36" s="4" t="str">
         <x:v>แยก finding จาก answer ถ้าต้อง track action</x:v>
@@ -2566,7 +2634,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J37" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K37" s="4" t="str">
         <x:v>ผูก safety_findings</x:v>
@@ -2601,7 +2669,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J38" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K38" s="4" t="str">
         <x:v>dashboard action</x:v>
@@ -2621,10 +2689,10 @@
         <x:v>บันทึก Fit to Drive/health check</x:v>
       </x:c>
       <x:c r="E39" s="4" t="str">
-        <x:v>Were OK</x:v>
+        <x:v>เมนูปิดอยู่</x:v>
       </x:c>
       <x:c r="F39" s="4" t="str">
-        <x:v>หลัง submit</x:v>
+        <x:v>ไม่เรียกจาก production UI</x:v>
       </x:c>
       <x:c r="G39" s="4" t="str">
         <x:v>User</x:v>
@@ -2636,10 +2704,10 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J39" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Disabled</x:v>
       </x:c>
       <x:c r="K39" s="4" t="str">
-        <x:v>รูป BP/Alc ใช้ uploads</x:v>
+        <x:v>Backend route คงไว้ แต่ /were-ok ถูกปิดใน menu config และไม่อยู่ใน scope การเชื่อม UI</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2656,10 +2724,10 @@
         <x:v>บันทึก Pre-trip Check</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>Were OK</x:v>
+        <x:v>เมนูปิดอยู่</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
-        <x:v>หลัง submit</x:v>
+        <x:v>ไม่เรียกจาก production UI</x:v>
       </x:c>
       <x:c r="G40" s="4" t="str">
         <x:v>User</x:v>
@@ -2671,10 +2739,10 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J40" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Disabled</x:v>
       </x:c>
       <x:c r="K40" s="4" t="str">
-        <x:v>payload JSON + activityId</x:v>
+        <x:v>Backend route คงไว้ แต่ /were-ok ถูกปิดใน menu config และไม่อยู่ใน scope การเชื่อม UI</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2691,10 +2759,10 @@
         <x:v>บันทึก KYT</x:v>
       </x:c>
       <x:c r="E41" s="4" t="str">
-        <x:v>Were OK</x:v>
+        <x:v>เมนูปิดอยู่</x:v>
       </x:c>
       <x:c r="F41" s="4" t="str">
-        <x:v>หลัง submit</x:v>
+        <x:v>ไม่เรียกจาก production UI</x:v>
       </x:c>
       <x:c r="G41" s="4" t="str">
         <x:v>User</x:v>
@@ -2706,10 +2774,10 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J41" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Disabled</x:v>
       </x:c>
       <x:c r="K41" s="4" t="str">
-        <x:v>รูป KYT ใช้ uploads</x:v>
+        <x:v>Backend route คงไว้ แต่ /were-ok ถูกปิดใน menu config และไม่อยู่ใน scope การเชื่อม UI</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2726,10 +2794,10 @@
         <x:v>บันทึก SOS</x:v>
       </x:c>
       <x:c r="E42" s="4" t="str">
-        <x:v>Were OK</x:v>
+        <x:v>เมนูปิดอยู่</x:v>
       </x:c>
       <x:c r="F42" s="4" t="str">
-        <x:v>หลัง submit</x:v>
+        <x:v>ไม่เรียกจาก production UI</x:v>
       </x:c>
       <x:c r="G42" s="4" t="str">
         <x:v>User</x:v>
@@ -2741,10 +2809,10 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J42" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Disabled</x:v>
       </x:c>
       <x:c r="K42" s="4" t="str">
-        <x:v>แจ้งเตือน admin</x:v>
+        <x:v>Backend route คงไว้ แต่ /were-ok ถูกปิดใน menu config และไม่อยู่ใน scope การเชื่อม UI</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -3091,7 +3159,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J52" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K52" s="4" t="str">
         <x:v>live/scheduled/closed</x:v>
@@ -3126,7 +3194,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J53" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K53" s="4" t="str">
         <x:v>แทน localStorage</x:v>
@@ -3161,7 +3229,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J54" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K54" s="4" t="str">
         <x:v>audit</x:v>
@@ -3196,7 +3264,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J55" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K55" s="4" t="str">
         <x:v>cache รายช่วงเวลา</x:v>
@@ -3231,7 +3299,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J56" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K56" s="4" t="str">
         <x:v>cache ได้</x:v>
@@ -3266,7 +3334,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J57" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K57" s="4" t="str">
         <x:v>transactional</x:v>
@@ -3301,7 +3369,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J58" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K58" s="4" t="str">
         <x:v>cache by date</x:v>
@@ -3371,7 +3439,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J60" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K60" s="4" t="str">
         <x:v>แทน in-memory/localStorage</x:v>
@@ -3406,9 +3474,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J61" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K61" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K61" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="4" t="str">
@@ -3439,7 +3509,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J62" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K62" s="4" t="str">
         <x:v>อาจ queue</x:v>
@@ -3474,7 +3544,7 @@
         <x:v>Upload size limit</x:v>
       </x:c>
       <x:c r="J63" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K63" s="4" t="str">
         <x:v>multipart/form-data</x:v>
@@ -3509,7 +3579,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J64" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K64" s="4" t="str">
         <x:v>ตรวจสิทธิ์</x:v>
@@ -3544,7 +3614,7 @@
         <x:v>File</x:v>
       </x:c>
       <x:c r="J65" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K65" s="4" t="str">
         <x:v>ใช้ signed URL/private URL</x:v>
@@ -3579,7 +3649,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J66" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K66" s="4" t="str">
         <x:v>soft delete + object lifecycle</x:v>
@@ -3614,7 +3684,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J67" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K67" s="4" t="str">
         <x:v>ลบรูปที่ไม่ถูกผูกกับ owner</x:v>
@@ -3649,7 +3719,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J68" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K68" s="4" t="str">
         <x:v>ใช้กับ company/division/fact/section</x:v>
@@ -3684,7 +3754,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J69" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K69" s="4" t="str">
         <x:v>ไม่โหลด tree ใหญ่ทุกครั้ง</x:v>
@@ -3719,9 +3789,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J70" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K70" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K70" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="4" t="str">
@@ -3752,7 +3824,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J71" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K71" s="4" t="str">
         <x:v>audit required</x:v>
@@ -3787,7 +3859,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J72" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K72" s="4" t="str">
         <x:v>audit required</x:v>
@@ -3822,7 +3894,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J73" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K73" s="4" t="str">
         <x:v>ต้องตรวจ child ก่อนลบ</x:v>
@@ -3857,7 +3929,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J74" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K74" s="4" t="str">
         <x:v>merge SSO + app profile</x:v>
@@ -3892,7 +3964,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J75" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K75" s="4" t="str">
         <x:v>profile image ใช้ mediaId</x:v>
@@ -3927,7 +3999,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J76" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K76" s="4" t="str">
         <x:v>ต้อง limit search</x:v>
@@ -3962,9 +4034,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J77" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K77" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K77" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="4" t="str">
@@ -3995,7 +4069,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J78" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K78" s="4" t="str">
         <x:v>audit required</x:v>
@@ -4030,9 +4104,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J79" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K79" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K79" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="4" t="str">
@@ -4063,9 +4139,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J80" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K80" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K80" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="4" t="str">
@@ -4096,9 +4174,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J81" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K81" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K81" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="4" t="str">
@@ -4129,9 +4209,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J82" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K82" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K82" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="4" t="str">
@@ -4162,7 +4244,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J83" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K83" s="4" t="str">
         <x:v>transactional</x:v>
@@ -4197,7 +4279,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J84" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K84" s="4" t="str">
         <x:v>transactional</x:v>
@@ -4214,13 +4296,13 @@
         <x:v>/api/location-imports</x:v>
       </x:c>
       <x:c r="D85" s="4" t="str">
-        <x:v>เริ่ม import/sync location master</x:v>
+        <x:v>upload/import master location file</x:v>
       </x:c>
       <x:c r="E85" s="4" t="str">
-        <x:v>Admin/Scheduled job</x:v>
+        <x:v>Admin</x:v>
       </x:c>
       <x:c r="F85" s="4" t="str">
-        <x:v>Admin import หรือ incremental RMR Plant sync</x:v>
+        <x:v>admin import DataOcean/Excel</x:v>
       </x:c>
       <x:c r="G85" s="4" t="str">
         <x:v>Admin</x:v>
@@ -4232,10 +4314,10 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J85" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K85" s="4" t="str">
-        <x:v>รองรับ body {source:"RMR_SSO_PLANT"}; SELECT-only แล้ว upsert CPAC mirror</x:v>
+        <x:v>สร้าง batch</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -4267,9 +4349,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J86" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K86" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K86" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="4" t="str">
@@ -4300,7 +4384,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J87" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K87" s="4" t="str">
         <x:v>รวม summary success/fail</x:v>
@@ -4335,7 +4419,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J88" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K88" s="4" t="str">
         <x:v>จำเป็นต้องแบ่งหน้า</x:v>
@@ -4370,9 +4454,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J89" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K89" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K89" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="4" t="str">
@@ -4403,7 +4489,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J90" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K90" s="4" t="str">
         <x:v>upsert locations</x:v>
@@ -4438,7 +4524,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J91" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K91" s="4" t="str">
         <x:v>spatial distance query</x:v>
@@ -4473,7 +4559,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J92" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K92" s="4" t="str">
         <x:v>ใช้ attachmentIds</x:v>
@@ -4508,9 +4594,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J93" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K93" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K93" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="4" t="str">
@@ -4541,7 +4629,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J94" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K94" s="4" t="str">
         <x:v>ใช้ aggregate/cache</x:v>
@@ -4576,9 +4664,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J95" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K95" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K95" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="4" t="str">
@@ -4609,7 +4699,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J96" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K96" s="4" t="str">
         <x:v>versioned</x:v>
@@ -4644,9 +4734,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J97" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K97" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K97" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="4" t="str">
@@ -4677,7 +4769,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J98" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K98" s="4" t="str">
         <x:v>lock questions</x:v>
@@ -4712,9 +4804,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J99" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K99" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K99" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="4" t="str">
@@ -4745,9 +4839,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J100" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K100" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K100" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="4" t="str">
@@ -4778,9 +4874,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J101" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K101" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K101" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="4" t="str">
@@ -4811,9 +4909,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J102" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K102" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K102" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="4" t="str">
@@ -4844,7 +4944,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J103" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K103" s="4" t="str">
         <x:v>soft disable if published</x:v>
@@ -4879,7 +4979,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J104" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K104" s="4" t="str">
         <x:v>server validates complete answers</x:v>
@@ -4914,7 +5014,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J105" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K105" s="4" t="str">
         <x:v>attachmentIds only</x:v>
@@ -4949,9 +5049,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J106" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K106" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K106" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="4" t="str">
@@ -4982,7 +5084,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J107" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K107" s="4" t="str">
         <x:v>cache by filter</x:v>
@@ -5017,9 +5119,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J108" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K108" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K108" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="4" t="str">
@@ -5050,9 +5154,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J109" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K109" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K109" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="4" t="str">
@@ -5083,9 +5189,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J110" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K110" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K110" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="4" t="str">
@@ -5116,7 +5224,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J111" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K111" s="4" t="str">
         <x:v>ใช้ได้หลาย module</x:v>
@@ -5151,9 +5259,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J112" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K112" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K112" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="4" t="str">
@@ -5184,7 +5294,7 @@
         <x:v>File</x:v>
       </x:c>
       <x:c r="J113" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K113" s="4" t="str">
         <x:v>signed URL or stream</x:v>
@@ -5219,9 +5329,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J114" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K114" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K114" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="4" t="str">
@@ -5252,7 +5364,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J115" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K115" s="4" t="str">
         <x:v>รวม action/media</x:v>
@@ -5287,9 +5399,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J116" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K116" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K116" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="4" t="str">
@@ -5320,9 +5434,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J117" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K117" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K117" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="4" t="str">
@@ -5353,7 +5469,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J118" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K118" s="4" t="str">
         <x:v>require evidence optional</x:v>
@@ -5388,9 +5504,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J119" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K119" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K119" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="4" t="str">
@@ -5421,9 +5539,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J120" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K120" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K120" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="4" t="str">
@@ -5454,7 +5574,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J121" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K121" s="4" t="str">
         <x:v>optional if moderation enabled</x:v>
@@ -5489,7 +5609,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J122" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K122" s="4" t="str">
         <x:v>with reason</x:v>
@@ -5524,9 +5644,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J123" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K123" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K123" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="4" t="str">
@@ -5557,9 +5679,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J124" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K124" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K124" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="4" t="str">
@@ -5593,7 +5717,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K125" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>DB-backed implementation</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -5628,7 +5752,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K126" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>DB-backed implementation</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -5663,7 +5787,7 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K127" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>DB-backed implementation</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -5695,7 +5819,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J128" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K128" s="4" t="str">
         <x:v>audit required</x:v>
@@ -5765,7 +5889,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J130" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K130" s="4" t="str">
         <x:v>reward image mediaId</x:v>
@@ -5800,9 +5924,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J131" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K131" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K131" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="4" t="str">
@@ -5833,7 +5959,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J132" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K132" s="4" t="str">
         <x:v>soft delete</x:v>
@@ -5868,9 +5994,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J133" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K133" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K133" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="4" t="str">
@@ -5901,7 +6029,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J134" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K134" s="4" t="str">
         <x:v>transaction-safe</x:v>
@@ -5936,7 +6064,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J135" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K135" s="4" t="str">
         <x:v>ledger</x:v>
@@ -5971,9 +6099,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J136" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K136" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K136" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="4" t="str">
@@ -6004,9 +6134,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J137" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K137" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K137" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="4" t="str">
@@ -6037,9 +6169,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J138" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K138" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K138" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="4" t="str">
@@ -6070,7 +6204,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J139" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K139" s="4" t="str">
         <x:v>soft disable</x:v>
@@ -6105,9 +6239,11 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J140" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K140" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K140" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="4" t="str">
@@ -6138,9 +6274,11 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="J141" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K141" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K141" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="4" t="str">
@@ -6171,7 +6309,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J142" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K142" s="4" t="str">
         <x:v>cache yearly</x:v>
@@ -6206,9 +6344,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J143" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K143" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K143" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="4" t="str">
@@ -6239,9 +6379,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J144" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K144" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K144" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="4" t="str">
@@ -6272,9 +6414,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J145" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K145" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K145" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="4" t="str">
@@ -6305,9 +6449,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J146" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K146" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K146" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="4" t="str">
@@ -6338,9 +6484,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J147" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K147" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K147" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="4" t="str">
@@ -6371,9 +6519,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J148" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K148" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K148" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="4" t="str">
@@ -6404,7 +6554,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J149" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K149" s="4" t="str">
         <x:v>ownerType/ownerId/linkType</x:v>
@@ -6439,9 +6589,11 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J150" s="10" t="str">
-        <x:v>Target</x:v>
-      </x:c>
-      <x:c r="K150" s="4"/>
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K150" s="4" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="4" t="str">
@@ -6472,7 +6624,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J151" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K151" s="4" t="str">
         <x:v>ตรวจสิทธิ์ตาม owner</x:v>
@@ -6507,7 +6659,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J152" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K152" s="4" t="str">
         <x:v>optional for scale</x:v>
@@ -6542,7 +6694,7 @@
         <x:v>Small</x:v>
       </x:c>
       <x:c r="J153" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K153" s="4" t="str">
         <x:v>verify object exists</x:v>
@@ -6550,60 +6702,60 @@
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="4" t="str">
-        <x:v>Audit</x:v>
+        <x:v>Safety Culture</x:v>
       </x:c>
       <x:c r="B154" s="4" t="str">
         <x:v>GET</x:v>
       </x:c>
       <x:c r="C154" s="4" t="str">
-        <x:v>/api/audit-logs?actor=&amp;entity=&amp;from=&amp;to=&amp;page=&amp;pageSize=</x:v>
+        <x:v>/api/safety-culture/teams</x:v>
       </x:c>
       <x:c r="D154" s="4" t="str">
-        <x:v>audit trail</x:v>
+        <x:v>อ่านทีมสำหรับหน้า admin leaderboard</x:v>
       </x:c>
       <x:c r="E154" s="4" t="str">
-        <x:v>Admin/Security</x:v>
+        <x:v>Admin Leaderboard</x:v>
       </x:c>
       <x:c r="F154" s="4" t="str">
-        <x:v>ตรวจสอบการแก้ไข</x:v>
+        <x:v>เปิดหน้าจัดการทีม</x:v>
       </x:c>
       <x:c r="G154" s="4" t="str">
-        <x:v>Admin</x:v>
+        <x:v>User</x:v>
       </x:c>
       <x:c r="H154" s="4" t="str">
-        <x:v>Required</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="I154" s="4" t="str">
-        <x:v>High</x:v>
+        <x:v>Small</x:v>
       </x:c>
       <x:c r="J154" s="10" t="str">
-        <x:v>Target</x:v>
+        <x:v>Existing</x:v>
       </x:c>
       <x:c r="K154" s="4" t="str">
-        <x:v>ห้ามเปิด public</x:v>
+        <x:v>อ่านจาก teams และ team_members</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="4" t="str">
-        <x:v>System</x:v>
+        <x:v>Safety Culture</x:v>
       </x:c>
       <x:c r="B155" s="4" t="str">
-        <x:v>GET</x:v>
+        <x:v>PUT</x:v>
       </x:c>
       <x:c r="C155" s="4" t="str">
-        <x:v>/api/health</x:v>
+        <x:v>/api/safety-culture/teams</x:v>
       </x:c>
       <x:c r="D155" s="4" t="str">
-        <x:v>health check</x:v>
+        <x:v>บันทึกรายการทีมสำหรับ leaderboard</x:v>
       </x:c>
       <x:c r="E155" s="4" t="str">
-        <x:v>Infra</x:v>
+        <x:v>Admin Leaderboard</x:v>
       </x:c>
       <x:c r="F155" s="4" t="str">
-        <x:v>monitoring</x:v>
+        <x:v>เมื่อ admin บันทึกทีม</x:v>
       </x:c>
       <x:c r="G155" s="4" t="str">
-        <x:v>Public/Internal</x:v>
+        <x:v>Admin</x:v>
       </x:c>
       <x:c r="H155" s="4" t="str">
         <x:v>No</x:v>
@@ -6615,42 +6767,182 @@
         <x:v>Existing</x:v>
       </x:c>
       <x:c r="K155" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+        <x:v>upsert/soft-delete teams</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="4" t="str">
-        <x:v>System</x:v>
+        <x:v>Settings</x:v>
       </x:c>
       <x:c r="B156" s="4" t="str">
         <x:v>GET</x:v>
       </x:c>
       <x:c r="C156" s="4" t="str">
+        <x:v>/api/safety-settings?key=</x:v>
+      </x:c>
+      <x:c r="D156" s="4" t="str">
+        <x:v>อ่านค่า safety settings จากฐานจริง</x:v>
+      </x:c>
+      <x:c r="E156" s="4" t="str">
+        <x:v>Safety Admin/DatePicker</x:v>
+      </x:c>
+      <x:c r="F156" s="4" t="str">
+        <x:v>โหลดหน้าหรือเปิด setting</x:v>
+      </x:c>
+      <x:c r="G156" s="4" t="str">
+        <x:v>User</x:v>
+      </x:c>
+      <x:c r="H156" s="4" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I156" s="4" t="str">
+        <x:v>Small</x:v>
+      </x:c>
+      <x:c r="J156" s="10" t="str">
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K156" s="4" t="str">
+        <x:v>ใช้ safety_settings ไม่ใช้ localStorage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="28" customHeight="1">
+      <x:c r="A157" s="14" t="str">
+        <x:v>Settings</x:v>
+      </x:c>
+      <x:c r="B157" s="14" t="str">
+        <x:v>PUT</x:v>
+      </x:c>
+      <x:c r="C157" s="14" t="str">
+        <x:v>/api/safety-settings</x:v>
+      </x:c>
+      <x:c r="D157" s="14" t="str">
+        <x:v>บันทึกค่า safety settings ลงฐานจริง</x:v>
+      </x:c>
+      <x:c r="E157" s="14" t="str">
+        <x:v>Safety Admin</x:v>
+      </x:c>
+      <x:c r="F157" s="14" t="str">
+        <x:v>เมื่อ admin save settings</x:v>
+      </x:c>
+      <x:c r="G157" s="14" t="str">
+        <x:v>Admin</x:v>
+      </x:c>
+      <x:c r="H157" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I157" s="14" t="str">
+        <x:v>Small</x:v>
+      </x:c>
+      <x:c r="J157" s="14" t="str">
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K157" s="14" t="str">
+        <x:v>upsert safety_settings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="28" customHeight="1">
+      <x:c r="A158" s="14" t="str">
+        <x:v>Audit</x:v>
+      </x:c>
+      <x:c r="B158" s="14" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C158" s="14" t="str">
+        <x:v>/api/audit-logs?actor=&amp;entity=&amp;from=&amp;to=&amp;page=&amp;pageSize=</x:v>
+      </x:c>
+      <x:c r="D158" s="14" t="str">
+        <x:v>audit trail</x:v>
+      </x:c>
+      <x:c r="E158" s="14" t="str">
+        <x:v>Admin/Security</x:v>
+      </x:c>
+      <x:c r="F158" s="14" t="str">
+        <x:v>ตรวจสอบการแก้ไข</x:v>
+      </x:c>
+      <x:c r="G158" s="14" t="str">
+        <x:v>Admin</x:v>
+      </x:c>
+      <x:c r="H158" s="14" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="I158" s="14" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="J158" s="14" t="str">
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K158" s="14" t="str">
+        <x:v>ห้ามเปิด public</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="28" customHeight="1">
+      <x:c r="A159" s="14" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="B159" s="14" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C159" s="14" t="str">
+        <x:v>/api/health</x:v>
+      </x:c>
+      <x:c r="D159" s="14" t="str">
+        <x:v>health check</x:v>
+      </x:c>
+      <x:c r="E159" s="14" t="str">
+        <x:v>Infra</x:v>
+      </x:c>
+      <x:c r="F159" s="14" t="str">
+        <x:v>monitoring</x:v>
+      </x:c>
+      <x:c r="G159" s="14" t="str">
+        <x:v>Public/Internal</x:v>
+      </x:c>
+      <x:c r="H159" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I159" s="14" t="str">
+        <x:v>Small</x:v>
+      </x:c>
+      <x:c r="J159" s="14" t="str">
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K159" s="14" t="str">
+        <x:v>DB-backed implementation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="28" customHeight="1">
+      <x:c r="A160" s="14" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="B160" s="14" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C160" s="14" t="str">
         <x:v>/api/version</x:v>
       </x:c>
-      <x:c r="D156" s="4" t="str">
+      <x:c r="D160" s="14" t="str">
         <x:v>app/api version</x:v>
       </x:c>
-      <x:c r="E156" s="4" t="str">
+      <x:c r="E160" s="14" t="str">
         <x:v>Infra/Debug</x:v>
       </x:c>
-      <x:c r="F156" s="4" t="str">
+      <x:c r="F160" s="14" t="str">
         <x:v>debug</x:v>
       </x:c>
-      <x:c r="G156" s="4" t="str">
+      <x:c r="G160" s="14" t="str">
         <x:v>Public/Internal</x:v>
       </x:c>
-      <x:c r="H156" s="4" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I156" s="4" t="str">
-        <x:v>Small</x:v>
-      </x:c>
-      <x:c r="J156" s="10" t="str">
-        <x:v>Existing</x:v>
-      </x:c>
-      <x:c r="K156" s="4" t="str">
-        <x:v>มี implementation ใน repo</x:v>
+      <x:c r="H160" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I160" s="14" t="str">
+        <x:v>Small</x:v>
+      </x:c>
+      <x:c r="J160" s="14" t="str">
+        <x:v>Existing</x:v>
+      </x:c>
+      <x:c r="K160" s="14" t="str">
+        <x:v>DB-backed implementation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7239,7 +7531,7 @@
         <x:v>feed posts</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
-        <x:v>posts, users, reactions, comments summary, media_asset_links</x:v>
+        <x:v>posts, users, reactions, comments summary, media_assets(owner_type, owner_id, link_type)</x:v>
       </x:c>
       <x:c r="E2" s="4" t="str">
         <x:v>cursor+limit</x:v>
@@ -7248,7 +7540,7 @@
         <x:v>thumbnail URLs only</x:v>
       </x:c>
       <x:c r="G2" s="4" t="str">
-        <x:v>แทน localStorage</x:v>
+        <x:v>อ่านจากฐานจริง; API fail แสดง error/empty state</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -7262,7 +7554,7 @@
         <x:v>create post</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>posts, media_asset_links, point_transactions</x:v>
+        <x:v>posts, media_assets(owner_type, owner_id, link_type), point_transactions</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
         <x:v>none</x:v>
@@ -7354,7 +7646,7 @@
         <x:v>campaign/activity config</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>culture_events</x:v>
+        <x:v>safety_safety_culture_events</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
         <x:v>page for admin</x:v>
@@ -7490,16 +7782,16 @@
         <x:v>Database</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>เก็บ metadata</x:v>
+        <x:v>เก็บ metadata และ owner link ใน media_assets</x:v>
       </x:c>
       <x:c r="C3" s="4" t="str">
-        <x:v>media_assets + media_asset_links</x:v>
+        <x:v>ใช้ owner_type, owner_id, link_type</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
         <x:v>ค้น/ผูก owner ได้โดยไม่แตะไฟล์ใหญ่</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
-        <x:v>id, url/key, mime, size, checksum, owner/link</x:v>
+        <x:v>ไม่มี media_asset_links แยกใน schema ปัจจุบัน</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -8011,6 +8303,142 @@
         <x:v>incremental upsert by source + external_key; missing source rows become INACTIVE</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>/api/safety-culture/events</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>safety_culture_events</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>users</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="str">
+        <x:v>กิจกรรมจริง ไม่เก็บ JSON ใน audit_logs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>/api/uploads, /api/media</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>media_assets</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>users</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="str">
+        <x:v>ไฟล์จริงใน storage; metadata/owner link ใน DB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>/api/exports</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>export_jobs</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>users</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="str">
+        <x:v>สร้างและติดตาม export job จริง</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="A25" s="14" t="str">
+        <x:v>/api/notifications/preferences</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>notification_preferences</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>users</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="str">
+        <x:v>ตั้งค่ารายผู้ใช้</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>/api/notifications/archive</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>archived_notifications</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>notifications, users</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>เก็บ archive จริง</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="14" t="str">
+        <x:v>/api/assessments/:id/attachments</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>assessment_attachments</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>assessment_runs, media_assets</x:v>
+      </x:c>
+      <x:c r="D27" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E27" s="14" t="str">
+        <x:v>หลักฐาน assessment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>/api/corrective-actions/:id/comments</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>corrective_action_comments</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>corrective_actions, users</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>ความคิดเห็น corrective action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>/api/safety-settings</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>safety_settings</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>users</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>Read/Write</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="str">
+        <x:v>Admin settings จริง</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>